<commit_message>
TC05: Add employee user vacancy candidate lifecycle
</commit_message>
<xml_diff>
--- a/test-cases/OrangeHRM_Test_Scenarios_and_Test_Cases.xlsx
+++ b/test-cases/OrangeHRM_Test_Scenarios_and_Test_Cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f3888815e5653624/Documents/Playwright Automation JS Project/playwright-js-framework-orangehrm/test-cases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="391" documentId="8_{91FEAD1C-4E00-41E5-AF4C-8C8A4231DF6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6365D500-1D36-4194-AA62-402AC264CD0E}"/>
+  <xr:revisionPtr revIDLastSave="466" documentId="8_{91FEAD1C-4E00-41E5-AF4C-8C8A4231DF6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E05BB8B-A4B2-438E-9070-C3ECC7A196EE}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D8EC82E4-2F5B-48CE-BD43-064CF51D43CB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D8EC82E4-2F5B-48CE-BD43-064CF51D43CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Scenarios" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="293">
   <si>
     <t>Scenario ID</t>
   </si>
@@ -781,6 +781,241 @@
   </si>
   <si>
     <t>Navigate to Leave → Apply Leave availability check → Leave type selection → Balance validation → Date entry → Comments → Leave submission → Overlap detection → Latest conflicting date identification → Next-date calculation → Automatic retry</t>
+  </si>
+  <si>
+    <t>TS05</t>
+  </si>
+  <si>
+    <t>Employee Lifecycle</t>
+  </si>
+  <si>
+    <t>Verify that an administrator can create an employee, retrieve the employee using the generated Employee ID, create and associate a system user with the employee, create a vacancy using the employee as Hiring Manager, create a candidate against the created vacancy, and verify the resulting associations.</t>
+  </si>
+  <si>
+    <t>TC05.01</t>
+  </si>
+  <si>
+    <t>Verify that the administrator can create a new employee for the lifecycle flow</t>
+  </si>
+  <si>
+    <t>User is successfully logged into the application and has access to PIM</t>
+  </si>
+  <si>
+    <t>1. Navigate to PIM
+2. Open Add Employee
+3. Enter employee details
+4. Click Save</t>
+  </si>
+  <si>
+    <t>Employee is created successfully and the employee details page is displayed</t>
+  </si>
+  <si>
+    <t>Verify that the generated Employee ID can be captured after employee creation</t>
+  </si>
+  <si>
+    <t>1. Access the employee details after creation
+2. Retrieve the generated Employee ID</t>
+  </si>
+  <si>
+    <t>A non-empty Employee ID is available for subsequent employee retrieval</t>
+  </si>
+  <si>
+    <t>TC05.02</t>
+  </si>
+  <si>
+    <t>Verify that the newly created employee can be retrieved using the generated Employee ID</t>
+  </si>
+  <si>
+    <t>Employee has been created and Employee ID has been captured</t>
+  </si>
+  <si>
+    <t>1. Navigate to Employee List
+2. Enter the Employee ID
+3. Search for the employee</t>
+  </si>
+  <si>
+    <t>The corresponding employee record is returned successfully</t>
+  </si>
+  <si>
+    <t>Verify that the administrator can create a system user associated with the created employee</t>
+  </si>
+  <si>
+    <t>Employee has been successfully created and retrieved</t>
+  </si>
+  <si>
+    <t>Employee name, unique username and password</t>
+  </si>
+  <si>
+    <t>1. Navigate to Admin → User Management
+2. Open Add User
+3. Select the created employee
+4. Enter username and password
+5. Save</t>
+  </si>
+  <si>
+    <t>System user is created successfully and is associated with the created employee</t>
+  </si>
+  <si>
+    <t>Verify that the created system user displays the expected employee association</t>
+  </si>
+  <si>
+    <t>System user has been created</t>
+  </si>
+  <si>
+    <t>Username and employee name</t>
+  </si>
+  <si>
+    <t>1. Search for the created system user
+2. Locate the user record</t>
+  </si>
+  <si>
+    <t>The system user record displays the expected employee name</t>
+  </si>
+  <si>
+    <t>TC05.03</t>
+  </si>
+  <si>
+    <t>TC05.04</t>
+  </si>
+  <si>
+    <t>TC05.05</t>
+  </si>
+  <si>
+    <t>TC05.06</t>
+  </si>
+  <si>
+    <t>Verify that the administrator can create a vacancy using the created employee as Hiring Manager</t>
+  </si>
+  <si>
+    <t>Employee and associated system user exist</t>
+  </si>
+  <si>
+    <t>Vacancy name, job title, description, employee as Hiring Manager, number of positions</t>
+  </si>
+  <si>
+    <t>Vacancy is created successfully with the created employee assigned as Hiring Manager</t>
+  </si>
+  <si>
+    <t>TC05.07</t>
+  </si>
+  <si>
+    <t>Verify that the created vacancy contains the expected Hiring Manager association</t>
+  </si>
+  <si>
+    <t>Vacancy has been successfully created</t>
+  </si>
+  <si>
+    <t>Vacancy name and employee name</t>
+  </si>
+  <si>
+    <t>Vacancy details are displayed correctly and the created employee is shown as the Hiring Manager</t>
+  </si>
+  <si>
+    <t>TC05.08</t>
+  </si>
+  <si>
+    <t>Verify that the administrator can create a candidate associated with the created vacancy</t>
+  </si>
+  <si>
+    <t>Created vacancy is available</t>
+  </si>
+  <si>
+    <t>Candidate name, email, created vacancy and resume</t>
+  </si>
+  <si>
+    <t>Candidate is created successfully and the Application Stage page is displayed</t>
+  </si>
+  <si>
+    <t>TC05.09</t>
+  </si>
+  <si>
+    <t>Verify that the created candidate is associated with the expected vacancy and Hiring Manager</t>
+  </si>
+  <si>
+    <t>Candidate has been successfully created</t>
+  </si>
+  <si>
+    <t>Candidate name, vacancy name and employee name</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Candidate displays the expected vacancy, Hiring Manager and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Application Initiated</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> status</t>
+    </r>
+  </si>
+  <si>
+    <t>TC05.10</t>
+  </si>
+  <si>
+    <t>Verify that the created candidate is displayed in the Candidates list with the expected associations</t>
+  </si>
+  <si>
+    <t>Candidate name, vacancy, Hiring Manager and status</t>
+  </si>
+  <si>
+    <t>Candidate record is displayed with the expected candidate name, vacancy, Hiring Manager and application status</t>
+  </si>
+  <si>
+    <t>1. Navigate to Recruitment → Vacancies
+2. Open Add Vacancy
+3. Enter vacancy details
+4. Select the created employee as Hiring Manager
+5. Save</t>
+  </si>
+  <si>
+    <t>1. Open the created vacancy
+2. Verify vacancy details
+3. Verify Hiring Manager</t>
+  </si>
+  <si>
+    <t>1. Navigate to Candidates
+2. Open Add Candidate
+3. Enter candidate details
+4. Select the created vacancy
+5. Upload resume
+6. Provide consent
+7. Save</t>
+  </si>
+  <si>
+    <t>1. Observe Application Stage
+2. Verify candidate name
+3. Verify vacancy
+4. Verify Hiring Manager
+5. Verify application status</t>
+  </si>
+  <si>
+    <t>1. Navigate back to Candidates
+2. Locate the created candidate
+3. Verify candidate details</t>
+  </si>
+  <si>
+    <t>TC05 - Verify employee can be associated with a system user, vacancy, and candidate</t>
+  </si>
+  <si>
+    <t>tests/employee-user-vacancy-lifecycle.spec.js</t>
+  </si>
+  <si>
+    <t>Login → Create Employee → Capture Employee ID → Retrieve Employee → Create System User → Verify System User → Create Vacancy using created employee as Hiring Manager → Verify Vacancy → Create Candidate using created vacancy → Verify Application Stage → Verify Candidate in Candidates list</t>
   </si>
 </sst>
 </file>
@@ -824,7 +1059,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -852,6 +1087,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -883,11 +1124,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -896,12 +1134,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -925,6 +1157,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -940,10 +1187,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1253,224 +1496,232 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="11" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="11" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="11" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
+    <row r="6" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
+      <c r="A16" s="1"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
+      <c r="A27" s="1"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
+      <c r="A28" s="1"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="2"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
+      <c r="A30" s="1"/>
+      <c r="B30" s="1"/>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1479,7 +1730,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA49C067-8F15-4F61-ABFB-E796688C4971}">
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.77734375" customWidth="1"/>
@@ -1493,1084 +1744,1218 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
     </row>
     <row r="2" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
     </row>
     <row r="3" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="2"/>
-      <c r="B3" s="7" t="s">
+      <c r="A3" s="11"/>
+      <c r="B3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2" t="s">
+      <c r="C3" s="11"/>
+      <c r="D3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
     </row>
     <row r="4" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
-      <c r="B4" s="7" t="s">
+      <c r="A4" s="11"/>
+      <c r="B4" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2" t="s">
+      <c r="C4" s="11"/>
+      <c r="D4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
     </row>
     <row r="5" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="2"/>
-      <c r="B5" s="7" t="s">
+      <c r="A5" s="11"/>
+      <c r="B5" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2" t="s">
+      <c r="C5" s="11"/>
+      <c r="D5" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
     </row>
     <row r="6" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="B6" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
     </row>
     <row r="7" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A7" s="2"/>
-      <c r="B7" s="8" t="s">
+      <c r="A7" s="11"/>
+      <c r="B7" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2" t="s">
+      <c r="C7" s="11"/>
+      <c r="D7" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
     </row>
     <row r="8" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="2"/>
-      <c r="B8" s="8" t="s">
+      <c r="A8" s="11"/>
+      <c r="B8" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2" t="s">
+      <c r="C8" s="11"/>
+      <c r="D8" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
     </row>
     <row r="9" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="8" t="s">
+      <c r="A9" s="11"/>
+      <c r="B9" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2" t="s">
+      <c r="C9" s="11"/>
+      <c r="D9" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
     </row>
     <row r="10" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="8" t="s">
+      <c r="A10" s="11"/>
+      <c r="B10" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2" t="s">
+      <c r="C10" s="11"/>
+      <c r="D10" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
     </row>
     <row r="11" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
-      <c r="L11" s="4"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
     </row>
     <row r="12" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="2"/>
-      <c r="B12" s="9" t="s">
+      <c r="A12" s="11"/>
+      <c r="B12" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2" t="s">
+      <c r="C12" s="11"/>
+      <c r="D12" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2" t="s">
+      <c r="F12" s="1"/>
+      <c r="G12" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
     </row>
     <row r="13" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="2"/>
-      <c r="B13" s="9" t="s">
+      <c r="A13" s="11"/>
+      <c r="B13" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2" t="s">
+      <c r="C13" s="11"/>
+      <c r="D13" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="G13" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="H13" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
-      <c r="L13" s="4"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
     </row>
     <row r="14" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="2"/>
-      <c r="B14" s="9" t="s">
+      <c r="A14" s="11"/>
+      <c r="B14" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2" t="s">
+      <c r="C14" s="11"/>
+      <c r="D14" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="G14" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="H14" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="4"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
     </row>
     <row r="15" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="2"/>
-      <c r="B15" s="9" t="s">
+      <c r="A15" s="11"/>
+      <c r="B15" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2" t="s">
+      <c r="C15" s="11"/>
+      <c r="D15" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="G15" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="H15" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
-      <c r="L15" s="4"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
     </row>
     <row r="16" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="2"/>
-      <c r="B16" s="9" t="s">
+      <c r="A16" s="11"/>
+      <c r="B16" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2" t="s">
+      <c r="C16" s="11"/>
+      <c r="D16" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="G16" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="H16" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
     </row>
     <row r="17" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="2"/>
-      <c r="B17" s="9" t="s">
+      <c r="A17" s="11"/>
+      <c r="B17" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2" t="s">
+      <c r="C17" s="11"/>
+      <c r="D17" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="F17" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="G17" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="H17" s="2" t="s">
+      <c r="H17" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
     </row>
     <row r="18" spans="1:12" ht="72" x14ac:dyDescent="0.3">
-      <c r="A18" s="2"/>
-      <c r="B18" s="9" t="s">
+      <c r="A18" s="11"/>
+      <c r="B18" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2" t="s">
+      <c r="C18" s="11"/>
+      <c r="D18" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="F18" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="G18" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="H18" s="2" t="s">
+      <c r="H18" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
     </row>
     <row r="19" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="2"/>
-      <c r="B19" s="9" t="s">
+      <c r="A19" s="11"/>
+      <c r="B19" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2" t="s">
+      <c r="C19" s="11"/>
+      <c r="D19" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F19" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="G19" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="H19" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="3"/>
     </row>
     <row r="20" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A20" s="2"/>
-      <c r="B20" s="9" t="s">
+      <c r="A20" s="11"/>
+      <c r="B20" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2" t="s">
+      <c r="C20" s="11"/>
+      <c r="D20" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="F20" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="G20" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="H20" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-      <c r="K20" s="4"/>
-      <c r="L20" s="4"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
     </row>
     <row r="21" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A21" s="2"/>
-      <c r="B21" s="9" t="s">
+      <c r="A21" s="11"/>
+      <c r="B21" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2" t="s">
+      <c r="C21" s="11"/>
+      <c r="D21" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="F21" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="G21" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="H21" s="2" t="s">
+      <c r="H21" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
-      <c r="K21" s="4"/>
-      <c r="L21" s="4"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
     </row>
     <row r="22" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="2"/>
-      <c r="B22" s="9" t="s">
+      <c r="A22" s="11"/>
+      <c r="B22" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2" t="s">
+      <c r="C22" s="11"/>
+      <c r="D22" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E22" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="F22" s="2" t="s">
+      <c r="F22" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="G22" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="H22" s="2" t="s">
+      <c r="H22" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
-      <c r="L22" s="4"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
     </row>
     <row r="23" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A23" s="2"/>
-      <c r="B23" s="9" t="s">
+      <c r="A23" s="11"/>
+      <c r="B23" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2" t="s">
+      <c r="C23" s="11"/>
+      <c r="D23" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="E23" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="F23" s="2" t="s">
+      <c r="F23" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="G23" s="2" t="s">
+      <c r="G23" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="H23" s="2" t="s">
+      <c r="H23" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
-      <c r="L23" s="4"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D24" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="E24" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="F24" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="G24" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="H24" s="2" t="s">
+      <c r="H24" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="I24" s="4"/>
-      <c r="J24" s="4"/>
-      <c r="K24" s="4"/>
-      <c r="L24" s="4"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A25" s="2"/>
-      <c r="B25" s="8" t="s">
+      <c r="A25" s="11"/>
+      <c r="B25" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2" t="s">
+      <c r="C25" s="11"/>
+      <c r="D25" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="E25" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="F25" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="G25" s="2" t="s">
+      <c r="G25" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="H25" s="2" t="s">
+      <c r="H25" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="I25" s="4"/>
-      <c r="J25" s="4"/>
-      <c r="K25" s="4"/>
-      <c r="L25" s="4"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
     </row>
     <row r="26" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="2"/>
-      <c r="B26" s="8" t="s">
+      <c r="A26" s="11"/>
+      <c r="B26" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2" t="s">
+      <c r="C26" s="11"/>
+      <c r="D26" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F26" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="G26" s="2" t="s">
+      <c r="G26" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="H26" s="2" t="s">
+      <c r="H26" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="I26" s="4"/>
-      <c r="J26" s="4"/>
-      <c r="K26" s="4"/>
-      <c r="L26" s="4"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
     </row>
     <row r="27" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A27" s="2"/>
-      <c r="B27" s="8" t="s">
+      <c r="A27" s="11"/>
+      <c r="B27" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2" t="s">
+      <c r="C27" s="11"/>
+      <c r="D27" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="F27" s="2" t="s">
+      <c r="F27" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="G27" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="H27" s="2" t="s">
+      <c r="H27" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
-      <c r="L27" s="4"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="3"/>
     </row>
     <row r="28" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A28" s="2"/>
-      <c r="B28" s="8" t="s">
+      <c r="A28" s="11"/>
+      <c r="B28" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2" t="s">
+      <c r="C28" s="11"/>
+      <c r="D28" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="E28" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="F28" s="2" t="s">
+      <c r="F28" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="G28" s="2" t="s">
+      <c r="G28" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="H28" s="2" t="s">
+      <c r="H28" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="I28" s="4"/>
-      <c r="J28" s="4"/>
-      <c r="K28" s="4"/>
-      <c r="L28" s="4"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
     </row>
     <row r="29" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A29" s="2"/>
-      <c r="B29" s="8" t="s">
+      <c r="A29" s="11"/>
+      <c r="B29" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2" t="s">
+      <c r="C29" s="11"/>
+      <c r="D29" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="E29" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="F29" s="2" t="s">
+      <c r="F29" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="G29" s="2" t="s">
+      <c r="G29" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="H29" s="2" t="s">
+      <c r="H29" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="I29" s="4"/>
-      <c r="J29" s="4"/>
-      <c r="K29" s="4"/>
-      <c r="L29" s="4"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
+      <c r="L29" s="3"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A30" s="2"/>
-      <c r="B30" s="8" t="s">
+      <c r="A30" s="11"/>
+      <c r="B30" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2" t="s">
+      <c r="C30" s="11"/>
+      <c r="D30" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="E30" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="F30" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="G30" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="H30" s="2" t="s">
+      <c r="H30" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="I30" s="4"/>
-      <c r="J30" s="4"/>
-      <c r="K30" s="4"/>
-      <c r="L30" s="4"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+      <c r="K30" s="3"/>
+      <c r="L30" s="3"/>
     </row>
     <row r="31" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A31" s="2"/>
-      <c r="B31" s="8" t="s">
+      <c r="A31" s="11"/>
+      <c r="B31" s="5" t="s">
         <v>210</v>
       </c>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2" t="s">
+      <c r="C31" s="11"/>
+      <c r="D31" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="E31" s="2" t="s">
+      <c r="E31" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="F31" s="2" t="s">
+      <c r="F31" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="G31" s="2" t="s">
+      <c r="G31" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="H31" s="2" t="s">
+      <c r="H31" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="I31" s="4"/>
-      <c r="J31" s="4"/>
-      <c r="K31" s="4"/>
-      <c r="L31" s="4"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="3"/>
+      <c r="K31" s="3"/>
+      <c r="L31" s="3"/>
     </row>
     <row r="32" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A32" s="2"/>
-      <c r="B32" s="8" t="s">
+      <c r="A32" s="11"/>
+      <c r="B32" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2" t="s">
+      <c r="C32" s="11"/>
+      <c r="D32" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="E32" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="F32" s="2" t="s">
+      <c r="F32" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="G32" s="2" t="s">
+      <c r="G32" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="H32" s="2" t="s">
+      <c r="H32" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="I32" s="4"/>
-      <c r="J32" s="4"/>
-      <c r="K32" s="4"/>
-      <c r="L32" s="4"/>
+      <c r="I32" s="3"/>
+      <c r="J32" s="3"/>
+      <c r="K32" s="3"/>
+      <c r="L32" s="3"/>
     </row>
     <row r="33" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A33" s="2"/>
-      <c r="B33" s="8" t="s">
+      <c r="A33" s="11"/>
+      <c r="B33" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2" t="s">
+      <c r="C33" s="11"/>
+      <c r="D33" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="E33" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="F33" s="2" t="s">
+      <c r="F33" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="G33" s="2" t="s">
+      <c r="G33" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="H33" s="2" t="s">
+      <c r="H33" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="I33" s="4"/>
-      <c r="J33" s="4"/>
-      <c r="K33" s="4"/>
-      <c r="L33" s="4"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="3"/>
+      <c r="K33" s="3"/>
+      <c r="L33" s="3"/>
     </row>
     <row r="34" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A34" s="2"/>
-      <c r="B34" s="8" t="s">
+      <c r="A34" s="11"/>
+      <c r="B34" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2" t="s">
+      <c r="C34" s="11"/>
+      <c r="D34" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="E34" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="F34" s="2" t="s">
+      <c r="F34" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="G34" s="2" t="s">
+      <c r="G34" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="H34" s="2" t="s">
+      <c r="H34" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="I34" s="4"/>
-      <c r="J34" s="4"/>
-      <c r="K34" s="4"/>
-      <c r="L34" s="4"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="3"/>
+      <c r="K34" s="3"/>
+      <c r="L34" s="3"/>
     </row>
     <row r="35" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A35" s="2"/>
-      <c r="B35" s="8" t="s">
+      <c r="A35" s="11"/>
+      <c r="B35" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2" t="s">
+      <c r="C35" s="11"/>
+      <c r="D35" s="1" t="s">
         <v>195</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="E35" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="F35" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="G35" s="2" t="s">
+      <c r="G35" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="H35" s="2" t="s">
+      <c r="H35" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="I35" s="4"/>
-      <c r="J35" s="4"/>
-      <c r="K35" s="4"/>
-      <c r="L35" s="4"/>
+      <c r="I35" s="3"/>
+      <c r="J35" s="3"/>
+      <c r="K35" s="3"/>
+      <c r="L35" s="3"/>
     </row>
     <row r="36" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A36" s="2"/>
-      <c r="B36" s="8" t="s">
+      <c r="A36" s="11"/>
+      <c r="B36" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2" t="s">
+      <c r="C36" s="11"/>
+      <c r="D36" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="E36" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="F36" s="2" t="s">
+      <c r="F36" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="G36" s="2" t="s">
+      <c r="G36" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="H36" s="2" t="s">
+      <c r="H36" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="I36" s="4"/>
-      <c r="J36" s="4"/>
-      <c r="K36" s="4"/>
-      <c r="L36" s="4"/>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A37" s="2"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-      <c r="G37" s="2"/>
-      <c r="H37" s="2"/>
-      <c r="I37" s="4"/>
-      <c r="J37" s="4"/>
-      <c r="K37" s="4"/>
-      <c r="L37" s="4"/>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A38" s="2"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
-      <c r="H38" s="2"/>
-      <c r="I38" s="4"/>
-      <c r="J38" s="4"/>
-      <c r="K38" s="4"/>
-      <c r="L38" s="4"/>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2"/>
-      <c r="G39" s="2"/>
-      <c r="H39" s="2"/>
-      <c r="I39" s="4"/>
-      <c r="J39" s="4"/>
-      <c r="K39" s="4"/>
-      <c r="L39" s="4"/>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A40" s="2"/>
-      <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
-      <c r="G40" s="2"/>
-      <c r="H40" s="2"/>
-      <c r="I40" s="4"/>
-      <c r="J40" s="4"/>
-      <c r="K40" s="4"/>
-      <c r="L40" s="4"/>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A41" s="2"/>
-      <c r="B41" s="2"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="2"/>
-      <c r="G41" s="2"/>
-      <c r="H41" s="2"/>
-      <c r="I41" s="4"/>
-      <c r="J41" s="4"/>
-      <c r="K41" s="4"/>
-      <c r="L41" s="4"/>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A42" s="2"/>
-      <c r="B42" s="2"/>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
-      <c r="F42" s="2"/>
-      <c r="G42" s="2"/>
-      <c r="H42" s="2"/>
-      <c r="I42" s="4"/>
-      <c r="J42" s="4"/>
-      <c r="K42" s="4"/>
-      <c r="L42" s="4"/>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A43" s="2"/>
-      <c r="B43" s="2"/>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
-      <c r="F43" s="2"/>
-      <c r="G43" s="2"/>
-      <c r="H43" s="2"/>
-      <c r="I43" s="4"/>
-      <c r="J43" s="4"/>
-      <c r="K43" s="4"/>
-      <c r="L43" s="4"/>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A44" s="2"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
-      <c r="F44" s="2"/>
-      <c r="G44" s="2"/>
-      <c r="H44" s="2"/>
-      <c r="I44" s="4"/>
-      <c r="J44" s="4"/>
-      <c r="K44" s="4"/>
-      <c r="L44" s="4"/>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A45" s="2"/>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-      <c r="G45" s="2"/>
-      <c r="H45" s="2"/>
-      <c r="I45" s="4"/>
-      <c r="J45" s="4"/>
-      <c r="K45" s="4"/>
-      <c r="L45" s="4"/>
+      <c r="I36" s="3"/>
+      <c r="J36" s="3"/>
+      <c r="K36" s="3"/>
+      <c r="L36" s="3"/>
+    </row>
+    <row r="37" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A37" s="14" t="s">
+        <v>232</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>235</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>233</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="I37" s="3"/>
+      <c r="J37" s="3"/>
+      <c r="K37" s="3"/>
+      <c r="L37" s="3"/>
+    </row>
+    <row r="38" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A38" s="11"/>
+      <c r="B38" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="C38" s="11"/>
+      <c r="D38" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="I38" s="3"/>
+      <c r="J38" s="3"/>
+      <c r="K38" s="3"/>
+      <c r="L38" s="3"/>
+    </row>
+    <row r="39" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A39" s="11"/>
+      <c r="B39" s="12" t="s">
+        <v>258</v>
+      </c>
+      <c r="C39" s="11"/>
+      <c r="D39" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="H39" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="I39" s="3"/>
+      <c r="J39" s="3"/>
+      <c r="K39" s="3"/>
+      <c r="L39" s="3"/>
+    </row>
+    <row r="40" spans="1:12" ht="72" x14ac:dyDescent="0.3">
+      <c r="A40" s="11"/>
+      <c r="B40" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="C40" s="11"/>
+      <c r="D40" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="I40" s="3"/>
+      <c r="J40" s="3"/>
+      <c r="K40" s="3"/>
+      <c r="L40" s="3"/>
+    </row>
+    <row r="41" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A41" s="11"/>
+      <c r="B41" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="C41" s="11"/>
+      <c r="D41" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="I41" s="3"/>
+      <c r="J41" s="3"/>
+      <c r="K41" s="3"/>
+      <c r="L41" s="3"/>
+    </row>
+    <row r="42" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A42" s="11"/>
+      <c r="B42" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="C42" s="11"/>
+      <c r="D42" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="H42" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="I42" s="3"/>
+      <c r="J42" s="3"/>
+      <c r="K42" s="3"/>
+      <c r="L42" s="3"/>
+    </row>
+    <row r="43" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A43" s="11"/>
+      <c r="B43" s="12" t="s">
+        <v>266</v>
+      </c>
+      <c r="C43" s="11"/>
+      <c r="D43" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="H43" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="I43" s="3"/>
+      <c r="J43" s="3"/>
+      <c r="K43" s="3"/>
+      <c r="L43" s="3"/>
+    </row>
+    <row r="44" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A44" s="11"/>
+      <c r="B44" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="C44" s="11"/>
+      <c r="D44" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="H44" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="I44" s="3"/>
+      <c r="J44" s="3"/>
+      <c r="K44" s="3"/>
+      <c r="L44" s="3"/>
+    </row>
+    <row r="45" spans="1:12" ht="72" x14ac:dyDescent="0.3">
+      <c r="A45" s="11"/>
+      <c r="B45" s="12" t="s">
+        <v>276</v>
+      </c>
+      <c r="C45" s="11"/>
+      <c r="D45" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="H45" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="I45" s="3"/>
+      <c r="J45" s="3"/>
+      <c r="K45" s="3"/>
+      <c r="L45" s="3"/>
+    </row>
+    <row r="46" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A46" s="15"/>
+      <c r="B46" s="12" t="s">
+        <v>281</v>
+      </c>
+      <c r="C46" s="15"/>
+      <c r="D46" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="H46" s="1" t="s">
+        <v>284</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -2591,166 +2976,176 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="8" t="s">
         <v>217</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="8" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="10" t="s">
         <v>225</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="1" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="10" t="s">
         <v>141</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="1" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
+    <row r="6" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>292</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="10"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
+      <c r="A16" s="7"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
test: add TC06-TC08 authorization and user validation coverage
</commit_message>
<xml_diff>
--- a/test-cases/OrangeHRM_Test_Scenarios_and_Test_Cases.xlsx
+++ b/test-cases/OrangeHRM_Test_Scenarios_and_Test_Cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f3888815e5653624/Documents/Playwright Automation JS Project/playwright-js-framework-orangehrm/test-cases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="466" documentId="8_{91FEAD1C-4E00-41E5-AF4C-8C8A4231DF6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E05BB8B-A4B2-438E-9070-C3ECC7A196EE}"/>
+  <xr:revisionPtr revIDLastSave="562" documentId="8_{91FEAD1C-4E00-41E5-AF4C-8C8A4231DF6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0DB3DED-899F-45BE-A1D7-82631AEB0BB0}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D8EC82E4-2F5B-48CE-BD43-064CF51D43CB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D8EC82E4-2F5B-48CE-BD43-064CF51D43CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Scenarios" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="403">
   <si>
     <t>Scenario ID</t>
   </si>
@@ -1017,12 +1017,400 @@
   <si>
     <t>Login → Create Employee → Capture Employee ID → Retrieve Employee → Create System User → Verify System User → Create Vacancy using created employee as Hiring Manager → Verify Vacancy → Create Candidate using created vacancy → Verify Application Stage → Verify Candidate in Candidates list</t>
   </si>
+  <si>
+    <t>TS06</t>
+  </si>
+  <si>
+    <t>Access Control / Authentication</t>
+  </si>
+  <si>
+    <t>Verify that an unauthenticated user attempting to access a protected page is redirected to the Login page and, after successful authentication, is returned to the originally requested protected page.</t>
+  </si>
+  <si>
+    <t>TS07</t>
+  </si>
+  <si>
+    <t>PIM - Employee &amp; User Management</t>
+  </si>
+  <si>
+    <t>Verify that an administrator can create an employee with login details, validate mandatory employee and password fields, authenticate using the newly created ESS account, and verify the account has the expected ESS-level access.</t>
+  </si>
+  <si>
+    <t>TS08</t>
+  </si>
+  <si>
+    <t>Verify that the application prevents creation of an employee account using a username that already exists.</t>
+  </si>
+  <si>
+    <t>TC06 - Verify unauthenticated user is redirected to login and returned to the originally requested protected page after authentication</t>
+  </si>
+  <si>
+    <t>tests/authentication-authorization.spec.js</t>
+  </si>
+  <si>
+    <t>Attempt to access a protected Admin page without authentication → Verify redirect to Login → Verify Login page → Authenticate with valid credentials → Verify return to originally requested protected page → Verify Admin module, Job context, and Job Categories page</t>
+  </si>
+  <si>
+    <t>TC07 - Verify employee creation with login details and ESS authentication</t>
+  </si>
+  <si>
+    <t>Login as Admin → Navigate to PIM → Add Employee → Validate mandatory Last Name → Enter Last Name → Enable Create Login Details → Verify default account configuration → Enter login credentials → Validate password mismatch → Correct password → Create employee and ESS account → Verify employee details → Capture Employee ID → Logout Admin → Login using newly created ESS credentials → Verify Dashboard → Verify logged-in employee identity → Verify Admin module is unavailable</t>
+  </si>
+  <si>
+    <t>TC08 - Verify duplicate username is rejected during employee account creation</t>
+  </si>
+  <si>
+    <t>Login as Admin → Create Employee #1 with valid login account → Verify successful creation → Return to Employee List → Add Employee #2 → Reuse Employee #1 username → Submit login details → Verify Username already exists validation</t>
+  </si>
+  <si>
+    <t>tests/employee-login-validation.spec.js</t>
+  </si>
+  <si>
+    <t>tests/duplicate-username-validation.spec.js</t>
+  </si>
+  <si>
+    <t>TC06.01</t>
+  </si>
+  <si>
+    <t>Access Control</t>
+  </si>
+  <si>
+    <t>Verify that an unauthenticated user is redirected to Login when accessing a protected page</t>
+  </si>
+  <si>
+    <t>User is not authenticated</t>
+  </si>
+  <si>
+    <t>Protected URL: /web/index.php/admin/jobCategory</t>
+  </si>
+  <si>
+    <t>1. Navigate directly to the protected Admin Job Categories URL</t>
+  </si>
+  <si>
+    <t>User is redirected to the Login page</t>
+  </si>
+  <si>
+    <t>Verify that the Login page is displayed after protected-page access is denied</t>
+  </si>
+  <si>
+    <t>User attempted to access protected page without authentication</t>
+  </si>
+  <si>
+    <t>1. Attempt to access protected Admin page 2. Observe redirected page</t>
+  </si>
+  <si>
+    <t>Login page and Login heading are displayed</t>
+  </si>
+  <si>
+    <t>Verify that the user is returned to the originally requested protected page after successful authentication</t>
+  </si>
+  <si>
+    <t>User has been redirected to Login from a protected page</t>
+  </si>
+  <si>
+    <t>Username: Admin / Password: admin123</t>
+  </si>
+  <si>
+    <t>1. Enter valid credentials 2. Submit login</t>
+  </si>
+  <si>
+    <t>User is authenticated and returned to the originally requested Admin Job Categories page</t>
+  </si>
+  <si>
+    <t>Verify that the originally requested protected page is displayed after authentication</t>
+  </si>
+  <si>
+    <t>User successfully authenticated after redirect</t>
+  </si>
+  <si>
+    <t>Job Categories page</t>
+  </si>
+  <si>
+    <t>1. Observe Admin breadcrumb 2. Observe Job context 3. Observe page title</t>
+  </si>
+  <si>
+    <t>Admin module, Job context, and Job Categories page are displayed</t>
+  </si>
+  <si>
+    <t>TC06.02</t>
+  </si>
+  <si>
+    <t>TC06.03</t>
+  </si>
+  <si>
+    <t>TC06.04</t>
+  </si>
+  <si>
+    <t>Verify that Last Name is mandatory when creating an employee</t>
+  </si>
+  <si>
+    <t>Admin is logged in and Add Employee page is displayed</t>
+  </si>
+  <si>
+    <t>First Name: Milo</t>
+  </si>
+  <si>
+    <t>1. Enter First Name 2. Leave Last Name empty 3. Click Save</t>
+  </si>
+  <si>
+    <t>Last Name required validation is displayed</t>
+  </si>
+  <si>
+    <t>Verify that login details can be enabled while creating an employee</t>
+  </si>
+  <si>
+    <t>Add Employee page is displayed with required employee details</t>
+  </si>
+  <si>
+    <t>Username: dynamically generated</t>
+  </si>
+  <si>
+    <t>1. Enter valid Last Name 2. Enable Create Login Details</t>
+  </si>
+  <si>
+    <t>Login-detail fields are displayed</t>
+  </si>
+  <si>
+    <t>Verify default ESS login configuration when login details are enabled</t>
+  </si>
+  <si>
+    <t>Create Login Details is enabled</t>
+  </si>
+  <si>
+    <t>1. Enable login details 2. Observe account configuration</t>
+  </si>
+  <si>
+    <t>Expected default login configuration is selected</t>
+  </si>
+  <si>
+    <t>Verify that mismatched passwords are rejected during account creation</t>
+  </si>
+  <si>
+    <t>Login details are enabled</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Password: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Test@12345</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> / Confirm Password: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Test@123456</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Enter mismatched passwords 2. Click Save</t>
+  </si>
+  <si>
+    <t>Password mismatch validation is displayed</t>
+  </si>
+  <si>
+    <t>Verify that an employee can be created with valid login details</t>
+  </si>
+  <si>
+    <t>Required employee and login details are valid</t>
+  </si>
+  <si>
+    <t>Valid dynamically generated employee/user data</t>
+  </si>
+  <si>
+    <t>1. Correct Confirm Password 2. Submit employee</t>
+  </si>
+  <si>
+    <t>Employee and ESS account are created successfully and Personal Details page is displayed</t>
+  </si>
+  <si>
+    <t>Verify that the generated Employee ID is assigned to the created employee</t>
+  </si>
+  <si>
+    <t>Dynamically generated Employee ID</t>
+  </si>
+  <si>
+    <t>1. Retrieve Employee ID from Personal Details page</t>
+  </si>
+  <si>
+    <t>A non-empty Employee ID is displayed</t>
+  </si>
+  <si>
+    <t>Verify that the newly created ESS user can authenticate successfully</t>
+  </si>
+  <si>
+    <t>Employee and ESS account were created successfully</t>
+  </si>
+  <si>
+    <t>Newly generated username/password</t>
+  </si>
+  <si>
+    <t>1. Logout Admin 2. Login using newly created ESS credentials</t>
+  </si>
+  <si>
+    <t>ESS user is authenticated and Dashboard is displayed</t>
+  </si>
+  <si>
+    <t>Verify that the authenticated ESS user is identified as the created employee</t>
+  </si>
+  <si>
+    <t>ESS user is logged in</t>
+  </si>
+  <si>
+    <t>Created employee display name</t>
+  </si>
+  <si>
+    <t>1. Observe user profile name</t>
+  </si>
+  <si>
+    <t>Logged-in profile displays the created employee's name</t>
+  </si>
+  <si>
+    <t>Verify that the ESS user cannot access the Admin module</t>
+  </si>
+  <si>
+    <t>ESS user is authenticated</t>
+  </si>
+  <si>
+    <t>1. Observe available navigation options</t>
+  </si>
+  <si>
+    <t>Admin module is not available to the ESS user</t>
+  </si>
+  <si>
+    <t>TC07.01</t>
+  </si>
+  <si>
+    <t>TC07.02</t>
+  </si>
+  <si>
+    <t>TC07.03</t>
+  </si>
+  <si>
+    <t>TC07.04</t>
+  </si>
+  <si>
+    <t>TC07.05</t>
+  </si>
+  <si>
+    <t>TC07.06</t>
+  </si>
+  <si>
+    <t>TC07.07</t>
+  </si>
+  <si>
+    <t>TC07.08</t>
+  </si>
+  <si>
+    <t>TC07.09</t>
+  </si>
+  <si>
+    <t>Verify that an employee can be created with a unique username</t>
+  </si>
+  <si>
+    <t>Admin is logged in and Add Employee page is available</t>
+  </si>
+  <si>
+    <t>Employee #1 + unique username</t>
+  </si>
+  <si>
+    <t>1. Create Employee #1 2. Enable login details 3. Enter unique username 4. Save</t>
+  </si>
+  <si>
+    <t>Employee is created successfully with the login account</t>
+  </si>
+  <si>
+    <t>Verify that an existing username cannot be reused for another employee account</t>
+  </si>
+  <si>
+    <t>Employee #1 with an active username already exists</t>
+  </si>
+  <si>
+    <t>Employee #2 + Employee #1 username</t>
+  </si>
+  <si>
+    <t>1. Return to Employee List 2. Open Add Employee 3. Create Employee #2 4. Enter existing username 5. Save</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Application rejects the username and displays </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Username already exists</t>
+    </r>
+  </si>
+  <si>
+    <t>Verify that duplicate username validation is displayed against the Username field</t>
+  </si>
+  <si>
+    <t>Duplicate username has been submitted</t>
+  </si>
+  <si>
+    <t>Existing username</t>
+  </si>
+  <si>
+    <t>1. Submit duplicate username 2. Observe Username field</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Username field enters error state and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Username already exists</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> is displayed</t>
+    </r>
+  </si>
+  <si>
+    <t>TC08.01</t>
+  </si>
+  <si>
+    <t>TC08.02</t>
+  </si>
+  <si>
+    <t>TC08.03</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1058,8 +1446,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1096,6 +1489,24 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1124,7 +1535,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1172,6 +1583,27 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1187,6 +1619,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1487,7 +1923,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E725BE47-B81F-452A-9F15-1B1E4ED10BFB}">
   <dimension ref="A1:D30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14.88671875" customWidth="1"/>
     <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
@@ -1495,7 +1931,7 @@
     <col min="4" max="4" width="17.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="40.049999999999997" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1509,7 +1945,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4">
       <c r="A2" s="10" t="s">
         <v>4</v>
       </c>
@@ -1523,7 +1959,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="28.8">
       <c r="A3" s="10" t="s">
         <v>37</v>
       </c>
@@ -1537,7 +1973,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="43.2">
       <c r="A4" s="10" t="s">
         <v>62</v>
       </c>
@@ -1551,7 +1987,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="43.2">
       <c r="A5" s="10" t="s">
         <v>141</v>
       </c>
@@ -1565,159 +2001,183 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:4" ht="57.6">
+      <c r="A6" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="10" t="s">
         <v>233</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="43.2">
+      <c r="A7" s="10" t="s">
+        <v>293</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>294</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="57.6">
+      <c r="A8" s="10" t="s">
+        <v>296</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>297</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="57.6">
+      <c r="A9" s="10" t="s">
+        <v>299</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>297</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -1730,8 +2190,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA49C067-8F15-4F61-ABFB-E796688C4971}">
-  <dimension ref="A1:L46"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:L62"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="11.77734375" customWidth="1"/>
     <col min="2" max="2" width="11.44140625" customWidth="1"/>
@@ -1743,7 +2203,7 @@
     <col min="8" max="8" width="39.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="40.049999999999997" customHeight="1">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -1773,7 +2233,7 @@
       <c r="K1" s="3"/>
       <c r="L1" s="3"/>
     </row>
-    <row r="2" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="43.2">
       <c r="A2" s="14" t="s">
         <v>4</v>
       </c>
@@ -1803,7 +2263,7 @@
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
     </row>
-    <row r="3" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="43.2">
       <c r="A3" s="11"/>
       <c r="B3" s="4" t="s">
         <v>20</v>
@@ -1829,7 +2289,7 @@
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
     </row>
-    <row r="4" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="43.2">
       <c r="A4" s="11"/>
       <c r="B4" s="4" t="s">
         <v>31</v>
@@ -1855,7 +2315,7 @@
       <c r="K4" s="3"/>
       <c r="L4" s="3"/>
     </row>
-    <row r="5" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="28.8">
       <c r="A5" s="11"/>
       <c r="B5" s="4" t="s">
         <v>32</v>
@@ -1881,7 +2341,7 @@
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
     </row>
-    <row r="6" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="43.2">
       <c r="A6" s="14" t="s">
         <v>37</v>
       </c>
@@ -1911,7 +2371,7 @@
       <c r="K6" s="3"/>
       <c r="L6" s="3"/>
     </row>
-    <row r="7" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="43.2">
       <c r="A7" s="11"/>
       <c r="B7" s="5" t="s">
         <v>48</v>
@@ -1937,7 +2397,7 @@
       <c r="K7" s="3"/>
       <c r="L7" s="3"/>
     </row>
-    <row r="8" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" ht="43.2">
       <c r="A8" s="11"/>
       <c r="B8" s="5" t="s">
         <v>49</v>
@@ -1963,7 +2423,7 @@
       <c r="K8" s="3"/>
       <c r="L8" s="3"/>
     </row>
-    <row r="9" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" ht="43.2">
       <c r="A9" s="11"/>
       <c r="B9" s="5" t="s">
         <v>50</v>
@@ -1989,7 +2449,7 @@
       <c r="K9" s="3"/>
       <c r="L9" s="3"/>
     </row>
-    <row r="10" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" ht="43.2">
       <c r="A10" s="11"/>
       <c r="B10" s="5" t="s">
         <v>51</v>
@@ -2015,7 +2475,7 @@
       <c r="K10" s="3"/>
       <c r="L10" s="3"/>
     </row>
-    <row r="11" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" ht="43.2">
       <c r="A11" s="14" t="s">
         <v>62</v>
       </c>
@@ -2045,7 +2505,7 @@
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
     </row>
-    <row r="12" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="28.8">
       <c r="A12" s="11"/>
       <c r="B12" s="6" t="s">
         <v>82</v>
@@ -2069,7 +2529,7 @@
       <c r="K12" s="3"/>
       <c r="L12" s="3"/>
     </row>
-    <row r="13" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" ht="57.6">
       <c r="A13" s="11"/>
       <c r="B13" s="6" t="s">
         <v>83</v>
@@ -2095,7 +2555,7 @@
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
     </row>
-    <row r="14" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" ht="57.6">
       <c r="A14" s="11"/>
       <c r="B14" s="6" t="s">
         <v>84</v>
@@ -2121,7 +2581,7 @@
       <c r="K14" s="3"/>
       <c r="L14" s="3"/>
     </row>
-    <row r="15" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" ht="43.2">
       <c r="A15" s="11"/>
       <c r="B15" s="6" t="s">
         <v>132</v>
@@ -2147,7 +2607,7 @@
       <c r="K15" s="3"/>
       <c r="L15" s="3"/>
     </row>
-    <row r="16" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" ht="57.6">
       <c r="A16" s="11"/>
       <c r="B16" s="6" t="s">
         <v>133</v>
@@ -2173,7 +2633,7 @@
       <c r="K16" s="3"/>
       <c r="L16" s="3"/>
     </row>
-    <row r="17" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" ht="57.6">
       <c r="A17" s="11"/>
       <c r="B17" s="6" t="s">
         <v>134</v>
@@ -2199,7 +2659,7 @@
       <c r="K17" s="3"/>
       <c r="L17" s="3"/>
     </row>
-    <row r="18" spans="1:12" ht="72" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" ht="72">
       <c r="A18" s="11"/>
       <c r="B18" s="6" t="s">
         <v>135</v>
@@ -2225,7 +2685,7 @@
       <c r="K18" s="3"/>
       <c r="L18" s="3"/>
     </row>
-    <row r="19" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" ht="57.6">
       <c r="A19" s="11"/>
       <c r="B19" s="6" t="s">
         <v>136</v>
@@ -2251,7 +2711,7 @@
       <c r="K19" s="3"/>
       <c r="L19" s="3"/>
     </row>
-    <row r="20" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" ht="86.4">
       <c r="A20" s="11"/>
       <c r="B20" s="6" t="s">
         <v>137</v>
@@ -2277,7 +2737,7 @@
       <c r="K20" s="3"/>
       <c r="L20" s="3"/>
     </row>
-    <row r="21" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" ht="43.2">
       <c r="A21" s="11"/>
       <c r="B21" s="6" t="s">
         <v>138</v>
@@ -2303,7 +2763,7 @@
       <c r="K21" s="3"/>
       <c r="L21" s="3"/>
     </row>
-    <row r="22" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" ht="57.6">
       <c r="A22" s="11"/>
       <c r="B22" s="6" t="s">
         <v>139</v>
@@ -2329,7 +2789,7 @@
       <c r="K22" s="3"/>
       <c r="L22" s="3"/>
     </row>
-    <row r="23" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" ht="28.8">
       <c r="A23" s="11"/>
       <c r="B23" s="6" t="s">
         <v>140</v>
@@ -2355,7 +2815,7 @@
       <c r="K23" s="3"/>
       <c r="L23" s="3"/>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12">
       <c r="A24" s="14" t="s">
         <v>141</v>
       </c>
@@ -2385,7 +2845,7 @@
       <c r="K24" s="3"/>
       <c r="L24" s="3"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12">
       <c r="A25" s="11"/>
       <c r="B25" s="5" t="s">
         <v>150</v>
@@ -2411,7 +2871,7 @@
       <c r="K25" s="3"/>
       <c r="L25" s="3"/>
     </row>
-    <row r="26" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" ht="57.6">
       <c r="A26" s="11"/>
       <c r="B26" s="5" t="s">
         <v>205</v>
@@ -2437,7 +2897,7 @@
       <c r="K26" s="3"/>
       <c r="L26" s="3"/>
     </row>
-    <row r="27" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" ht="28.8">
       <c r="A27" s="11"/>
       <c r="B27" s="5" t="s">
         <v>206</v>
@@ -2463,7 +2923,7 @@
       <c r="K27" s="3"/>
       <c r="L27" s="3"/>
     </row>
-    <row r="28" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" ht="28.8">
       <c r="A28" s="11"/>
       <c r="B28" s="5" t="s">
         <v>207</v>
@@ -2489,7 +2949,7 @@
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
     </row>
-    <row r="29" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" ht="28.8">
       <c r="A29" s="11"/>
       <c r="B29" s="5" t="s">
         <v>208</v>
@@ -2515,7 +2975,7 @@
       <c r="K29" s="3"/>
       <c r="L29" s="3"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12">
       <c r="A30" s="11"/>
       <c r="B30" s="5" t="s">
         <v>209</v>
@@ -2541,7 +3001,7 @@
       <c r="K30" s="3"/>
       <c r="L30" s="3"/>
     </row>
-    <row r="31" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" ht="28.8">
       <c r="A31" s="11"/>
       <c r="B31" s="5" t="s">
         <v>210</v>
@@ -2567,7 +3027,7 @@
       <c r="K31" s="3"/>
       <c r="L31" s="3"/>
     </row>
-    <row r="32" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" ht="28.8">
       <c r="A32" s="11"/>
       <c r="B32" s="5" t="s">
         <v>211</v>
@@ -2593,7 +3053,7 @@
       <c r="K32" s="3"/>
       <c r="L32" s="3"/>
     </row>
-    <row r="33" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" ht="43.2">
       <c r="A33" s="11"/>
       <c r="B33" s="5" t="s">
         <v>212</v>
@@ -2619,7 +3079,7 @@
       <c r="K33" s="3"/>
       <c r="L33" s="3"/>
     </row>
-    <row r="34" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" ht="28.8">
       <c r="A34" s="11"/>
       <c r="B34" s="5" t="s">
         <v>213</v>
@@ -2645,7 +3105,7 @@
       <c r="K34" s="3"/>
       <c r="L34" s="3"/>
     </row>
-    <row r="35" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" ht="43.2">
       <c r="A35" s="11"/>
       <c r="B35" s="5" t="s">
         <v>214</v>
@@ -2671,7 +3131,7 @@
       <c r="K35" s="3"/>
       <c r="L35" s="3"/>
     </row>
-    <row r="36" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" ht="43.2">
       <c r="A36" s="11"/>
       <c r="B36" s="5" t="s">
         <v>215</v>
@@ -2697,7 +3157,7 @@
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
     </row>
-    <row r="37" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" ht="57.6">
       <c r="A37" s="14" t="s">
         <v>232</v>
       </c>
@@ -2727,7 +3187,7 @@
       <c r="K37" s="3"/>
       <c r="L37" s="3"/>
     </row>
-    <row r="38" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" ht="43.2">
       <c r="A38" s="11"/>
       <c r="B38" s="12" t="s">
         <v>243</v>
@@ -2753,7 +3213,7 @@
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
     </row>
-    <row r="39" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" ht="43.2">
       <c r="A39" s="11"/>
       <c r="B39" s="12" t="s">
         <v>258</v>
@@ -2779,7 +3239,7 @@
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
     </row>
-    <row r="40" spans="1:12" ht="72" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" ht="72">
       <c r="A40" s="11"/>
       <c r="B40" s="12" t="s">
         <v>259</v>
@@ -2805,7 +3265,7 @@
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
     </row>
-    <row r="41" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" ht="43.2">
       <c r="A41" s="11"/>
       <c r="B41" s="12" t="s">
         <v>260</v>
@@ -2831,7 +3291,7 @@
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
     </row>
-    <row r="42" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" ht="86.4">
       <c r="A42" s="11"/>
       <c r="B42" s="12" t="s">
         <v>261</v>
@@ -2857,7 +3317,7 @@
       <c r="K42" s="3"/>
       <c r="L42" s="3"/>
     </row>
-    <row r="43" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" ht="43.2">
       <c r="A43" s="11"/>
       <c r="B43" s="12" t="s">
         <v>266</v>
@@ -2883,7 +3343,7 @@
       <c r="K43" s="3"/>
       <c r="L43" s="3"/>
     </row>
-    <row r="44" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" ht="100.8">
       <c r="A44" s="11"/>
       <c r="B44" s="12" t="s">
         <v>271</v>
@@ -2909,7 +3369,7 @@
       <c r="K44" s="3"/>
       <c r="L44" s="3"/>
     </row>
-    <row r="45" spans="1:12" ht="72" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" ht="72">
       <c r="A45" s="11"/>
       <c r="B45" s="12" t="s">
         <v>276</v>
@@ -2935,7 +3395,7 @@
       <c r="K45" s="3"/>
       <c r="L45" s="3"/>
     </row>
-    <row r="46" spans="1:12" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" ht="43.2">
       <c r="A46" s="15"/>
       <c r="B46" s="12" t="s">
         <v>281</v>
@@ -2955,6 +3415,370 @@
       </c>
       <c r="H46" s="1" t="s">
         <v>284</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" ht="43.2">
+      <c r="A47" s="18" t="s">
+        <v>293</v>
+      </c>
+      <c r="B47" s="19" t="s">
+        <v>310</v>
+      </c>
+      <c r="C47" s="20" t="s">
+        <v>311</v>
+      </c>
+      <c r="D47" s="21" t="s">
+        <v>312</v>
+      </c>
+      <c r="E47" s="21" t="s">
+        <v>313</v>
+      </c>
+      <c r="F47" s="21" t="s">
+        <v>314</v>
+      </c>
+      <c r="G47" s="21" t="s">
+        <v>315</v>
+      </c>
+      <c r="H47" s="21" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" ht="43.2">
+      <c r="A48" s="11"/>
+      <c r="B48" s="19" t="s">
+        <v>331</v>
+      </c>
+      <c r="C48" s="11"/>
+      <c r="D48" s="17" t="s">
+        <v>317</v>
+      </c>
+      <c r="E48" s="17" t="s">
+        <v>318</v>
+      </c>
+      <c r="F48" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="G48" s="17" t="s">
+        <v>319</v>
+      </c>
+      <c r="H48" s="17" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="57.6">
+      <c r="A49" s="11"/>
+      <c r="B49" s="19" t="s">
+        <v>332</v>
+      </c>
+      <c r="C49" s="11"/>
+      <c r="D49" s="17" t="s">
+        <v>321</v>
+      </c>
+      <c r="E49" s="17" t="s">
+        <v>322</v>
+      </c>
+      <c r="F49" s="17" t="s">
+        <v>323</v>
+      </c>
+      <c r="G49" s="17" t="s">
+        <v>324</v>
+      </c>
+      <c r="H49" s="17" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="43.2">
+      <c r="A50" s="11"/>
+      <c r="B50" s="19" t="s">
+        <v>333</v>
+      </c>
+      <c r="C50" s="11"/>
+      <c r="D50" s="17" t="s">
+        <v>326</v>
+      </c>
+      <c r="E50" s="17" t="s">
+        <v>327</v>
+      </c>
+      <c r="F50" s="17" t="s">
+        <v>328</v>
+      </c>
+      <c r="G50" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="H50" s="17" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="43.2">
+      <c r="A51" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="B51" s="22" t="s">
+        <v>376</v>
+      </c>
+      <c r="C51" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="D51" s="17" t="s">
+        <v>334</v>
+      </c>
+      <c r="E51" s="17" t="s">
+        <v>335</v>
+      </c>
+      <c r="F51" s="17" t="s">
+        <v>336</v>
+      </c>
+      <c r="G51" s="17" t="s">
+        <v>337</v>
+      </c>
+      <c r="H51" s="17" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" ht="43.2">
+      <c r="A52" s="11"/>
+      <c r="B52" s="22" t="s">
+        <v>377</v>
+      </c>
+      <c r="C52" s="11"/>
+      <c r="D52" s="17" t="s">
+        <v>339</v>
+      </c>
+      <c r="E52" s="17" t="s">
+        <v>340</v>
+      </c>
+      <c r="F52" s="17" t="s">
+        <v>341</v>
+      </c>
+      <c r="G52" s="17" t="s">
+        <v>342</v>
+      </c>
+      <c r="H52" s="17" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" ht="43.2">
+      <c r="A53" s="11"/>
+      <c r="B53" s="22" t="s">
+        <v>378</v>
+      </c>
+      <c r="C53" s="11"/>
+      <c r="D53" s="17" t="s">
+        <v>344</v>
+      </c>
+      <c r="E53" s="17" t="s">
+        <v>345</v>
+      </c>
+      <c r="F53" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="G53" s="17" t="s">
+        <v>346</v>
+      </c>
+      <c r="H53" s="17" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" ht="43.2">
+      <c r="A54" s="11"/>
+      <c r="B54" s="22" t="s">
+        <v>379</v>
+      </c>
+      <c r="C54" s="11"/>
+      <c r="D54" s="17" t="s">
+        <v>348</v>
+      </c>
+      <c r="E54" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="F54" s="17" t="s">
+        <v>350</v>
+      </c>
+      <c r="G54" s="17" t="s">
+        <v>351</v>
+      </c>
+      <c r="H54" s="17" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" ht="43.2">
+      <c r="A55" s="11"/>
+      <c r="B55" s="22" t="s">
+        <v>380</v>
+      </c>
+      <c r="C55" s="11"/>
+      <c r="D55" s="17" t="s">
+        <v>353</v>
+      </c>
+      <c r="E55" s="17" t="s">
+        <v>354</v>
+      </c>
+      <c r="F55" s="17" t="s">
+        <v>355</v>
+      </c>
+      <c r="G55" s="17" t="s">
+        <v>356</v>
+      </c>
+      <c r="H55" s="17" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" ht="43.2">
+      <c r="A56" s="11"/>
+      <c r="B56" s="22" t="s">
+        <v>381</v>
+      </c>
+      <c r="C56" s="11"/>
+      <c r="D56" s="17" t="s">
+        <v>358</v>
+      </c>
+      <c r="E56" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="F56" s="17" t="s">
+        <v>359</v>
+      </c>
+      <c r="G56" s="17" t="s">
+        <v>360</v>
+      </c>
+      <c r="H56" s="17" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" ht="28.8">
+      <c r="A57" s="11"/>
+      <c r="B57" s="22" t="s">
+        <v>382</v>
+      </c>
+      <c r="C57" s="11"/>
+      <c r="D57" s="17" t="s">
+        <v>362</v>
+      </c>
+      <c r="E57" s="17" t="s">
+        <v>363</v>
+      </c>
+      <c r="F57" s="17" t="s">
+        <v>364</v>
+      </c>
+      <c r="G57" s="17" t="s">
+        <v>365</v>
+      </c>
+      <c r="H57" s="17" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" ht="43.2">
+      <c r="A58" s="11"/>
+      <c r="B58" s="22" t="s">
+        <v>383</v>
+      </c>
+      <c r="C58" s="11"/>
+      <c r="D58" s="17" t="s">
+        <v>367</v>
+      </c>
+      <c r="E58" s="17" t="s">
+        <v>368</v>
+      </c>
+      <c r="F58" s="17" t="s">
+        <v>369</v>
+      </c>
+      <c r="G58" s="17" t="s">
+        <v>370</v>
+      </c>
+      <c r="H58" s="17" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" ht="28.8">
+      <c r="A59" s="11"/>
+      <c r="B59" s="22" t="s">
+        <v>384</v>
+      </c>
+      <c r="C59" s="11"/>
+      <c r="D59" s="17" t="s">
+        <v>372</v>
+      </c>
+      <c r="E59" s="17" t="s">
+        <v>373</v>
+      </c>
+      <c r="F59" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="G59" s="17" t="s">
+        <v>374</v>
+      </c>
+      <c r="H59" s="17" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" ht="28.8">
+      <c r="A60" s="14" t="s">
+        <v>299</v>
+      </c>
+      <c r="B60" s="23" t="s">
+        <v>400</v>
+      </c>
+      <c r="C60" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="D60" s="17" t="s">
+        <v>385</v>
+      </c>
+      <c r="E60" s="17" t="s">
+        <v>386</v>
+      </c>
+      <c r="F60" s="17" t="s">
+        <v>387</v>
+      </c>
+      <c r="G60" s="17" t="s">
+        <v>388</v>
+      </c>
+      <c r="H60" s="17" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" ht="43.2">
+      <c r="A61" s="11"/>
+      <c r="B61" s="23" t="s">
+        <v>401</v>
+      </c>
+      <c r="C61" s="11"/>
+      <c r="D61" s="17" t="s">
+        <v>390</v>
+      </c>
+      <c r="E61" s="17" t="s">
+        <v>391</v>
+      </c>
+      <c r="F61" s="17" t="s">
+        <v>392</v>
+      </c>
+      <c r="G61" s="17" t="s">
+        <v>393</v>
+      </c>
+      <c r="H61" s="17" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" ht="43.2">
+      <c r="A62" s="11"/>
+      <c r="B62" s="23" t="s">
+        <v>402</v>
+      </c>
+      <c r="C62" s="11"/>
+      <c r="D62" s="17" t="s">
+        <v>395</v>
+      </c>
+      <c r="E62" s="17" t="s">
+        <v>396</v>
+      </c>
+      <c r="F62" s="17" t="s">
+        <v>397</v>
+      </c>
+      <c r="G62" s="17" t="s">
+        <v>398</v>
+      </c>
+      <c r="H62" s="17" t="s">
+        <v>399</v>
       </c>
     </row>
   </sheetData>
@@ -2966,7 +3790,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0ECDC79D-EE75-45A2-99C1-C7DF3481F80E}">
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="15.44140625" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -2975,7 +3799,7 @@
     <col min="5" max="5" width="46.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -2992,7 +3816,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="43.2">
       <c r="A2" s="10" t="s">
         <v>4</v>
       </c>
@@ -3009,7 +3833,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="43.2">
       <c r="A3" s="10" t="s">
         <v>37</v>
       </c>
@@ -3026,7 +3850,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="129.6">
       <c r="A4" s="10" t="s">
         <v>62</v>
       </c>
@@ -3043,7 +3867,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="72">
       <c r="A5" s="10" t="s">
         <v>141</v>
       </c>
@@ -3060,11 +3884,11 @@
         <v>231</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:5" ht="86.4">
+      <c r="A6" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="10" t="s">
         <v>233</v>
       </c>
       <c r="C6" s="1" t="s">
@@ -3077,70 +3901,100 @@
         <v>292</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" ht="86.4">
+      <c r="A7" s="10" t="s">
+        <v>293</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>294</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="144">
+      <c r="A8" s="10" t="s">
+        <v>296</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>297</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="72">
+      <c r="A9" s="10" t="s">
+        <v>299</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>297</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5">
       <c r="A15" s="7"/>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
       <c r="E15" s="7"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5">
       <c r="A16" s="7"/>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>

</xml_diff>

<commit_message>
Add accessibility regression baseline and stabilize PIM tests
</commit_message>
<xml_diff>
--- a/test-cases/OrangeHRM_Test_Scenarios_and_Test_Cases.xlsx
+++ b/test-cases/OrangeHRM_Test_Scenarios_and_Test_Cases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f3888815e5653624/Documents/Playwright Automation JS Project/playwright-js-framework-orangehrm/test-cases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="562" documentId="8_{91FEAD1C-4E00-41E5-AF4C-8C8A4231DF6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0DB3DED-899F-45BE-A1D7-82631AEB0BB0}"/>
+  <xr:revisionPtr revIDLastSave="689" documentId="8_{91FEAD1C-4E00-41E5-AF4C-8C8A4231DF6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F73C89B9-2BF3-44C1-BCE8-35FD4D50692C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D8EC82E4-2F5B-48CE-BD43-064CF51D43CB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D8EC82E4-2F5B-48CE-BD43-064CF51D43CB}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Scenarios" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="403">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="460">
   <si>
     <t>Scenario ID</t>
   </si>
@@ -1404,6 +1404,177 @@
   </si>
   <si>
     <t>TC08.03</t>
+  </si>
+  <si>
+    <t>TS09</t>
+  </si>
+  <si>
+    <t>Verify that the Login page is scanned for accessibility violations against the configured axe-core rules, and that detected violations and scan results are reported.</t>
+  </si>
+  <si>
+    <t>TS10</t>
+  </si>
+  <si>
+    <t>Verify that the Dashboard is scanned for accessibility violations after successful authentication and that scan results are reported.</t>
+  </si>
+  <si>
+    <t>TS11</t>
+  </si>
+  <si>
+    <t>Verify that the PIM Employee List page is scanned for accessibility violations and that detected issues are included in the accessibility reports.</t>
+  </si>
+  <si>
+    <t>TS12</t>
+  </si>
+  <si>
+    <t>Verify that the System Users page is scanned for accessibility violations and that scan results are reported.</t>
+  </si>
+  <si>
+    <t>TS13</t>
+  </si>
+  <si>
+    <t>Verify that the Add User page is scanned for accessibility violations and that detected issues are included in the accessibility reports.</t>
+  </si>
+  <si>
+    <t>Accessibility-Login</t>
+  </si>
+  <si>
+    <t>Accessibility-Dashboard</t>
+  </si>
+  <si>
+    <t>Accessibility-Employee List</t>
+  </si>
+  <si>
+    <t>Accessibility-System Users</t>
+  </si>
+  <si>
+    <t>Accessibility-Add User</t>
+  </si>
+  <si>
+    <t>TC09 – Run accessibility scan on Login page</t>
+  </si>
+  <si>
+    <t>tests/accessibility.spec.js</t>
+  </si>
+  <si>
+    <t>Navigate to Login → Load the page → Execute axe-core accessibility scan → Collect violations, passes, and incomplete checks → Generate detailed HTML report → Record summary results</t>
+  </si>
+  <si>
+    <t>Accessibility_Dashboard</t>
+  </si>
+  <si>
+    <t>TC10 – Run accessibility scan on Dashboard page</t>
+  </si>
+  <si>
+    <t>Login as Admin → Verify Dashboard is displayed → Execute axe-core accessibility scan → Collect scan results → Generate detailed HTML report → Record summary results</t>
+  </si>
+  <si>
+    <t>TC11 – Run accessibility scan on Employee List page</t>
+  </si>
+  <si>
+    <t>Login as Admin → Navigate to PIM → Open Employee List → Verify target page is loaded → Execute axe-core accessibility scan → Generate detailed HTML report → Record summary results</t>
+  </si>
+  <si>
+    <t>TC12 – Run accessibility scan on System Users page</t>
+  </si>
+  <si>
+    <t>Login as Admin → Navigate to Admin → Open User Management/System Users → Verify target page is loaded → Execute axe-core accessibility scan → Generate detailed HTML report → Record summary results</t>
+  </si>
+  <si>
+    <t>TC13 – Run accessibility scan on Add User page</t>
+  </si>
+  <si>
+    <t>Login as Admin → Navigate to Admin → Open User Management → Select Add User → Verify target page is loaded → Execute axe-core accessibility scan → Generate detailed HTML report → Record summary results</t>
+  </si>
+  <si>
+    <t>Verify that the Login page is scanned for accessibility violations.</t>
+  </si>
+  <si>
+    <t>TS09.1</t>
+  </si>
+  <si>
+    <t>OrangeHRM application is accessible, and the Login page can be loaded without authentication.</t>
+  </si>
+  <si>
+    <t>Login page URL; configured axe-core accessibility rules.</t>
+  </si>
+  <si>
+    <t>1. Navigate to the OrangeHRM Login page. 2. Verify that the Login page is loaded. 3. Execute the axe-core accessibility scan. 4. Collect violations, passes, and incomplete checks. 5. Generate the detailed HTML report and update the accessibility summary.</t>
+  </si>
+  <si>
+    <t>The scan completes, detected violations and incomplete checks are captured, and the detailed report and summary results are generated.</t>
+  </si>
+  <si>
+    <t>Verify that the Dashboard is scanned for accessibility violations after successful authentication.</t>
+  </si>
+  <si>
+    <t>TS10.1</t>
+  </si>
+  <si>
+    <t>Valid administrator credentials are available, and the OrangeHRM application is accessible.</t>
+  </si>
+  <si>
+    <t>Username: Admin; Password: admin123; configured axe-core accessibility rules.</t>
+  </si>
+  <si>
+    <t>1. Navigate to the Login page. 2. Authenticate using valid administrator credentials. 3. Verify that the Dashboard is displayed. 4. Execute the axe-core accessibility scan. 5. Collect scan results. 6. Generate the detailed HTML report and update the accessibility summary.</t>
+  </si>
+  <si>
+    <t>The Dashboard scan completes successfully, scan results are recorded, and the detailed report and summary are generated.</t>
+  </si>
+  <si>
+    <t>TS11.1</t>
+  </si>
+  <si>
+    <t>Verify that the PIM Employee List page is scanned for accessibility violations.</t>
+  </si>
+  <si>
+    <t>Valid administrator credentials are available, and the administrator can access the PIM module.</t>
+  </si>
+  <si>
+    <t>Administrator credentials; Employee List page; configured axe-core accessibility rules.</t>
+  </si>
+  <si>
+    <t>1. Log in as Admin. 2. Navigate to the PIM module. 3. Open Employee List. 4. Verify that the Employee List page is displayed. 5. Execute the axe-core accessibility scan. 6. Record violations, passes, and incomplete checks. 7. Generate the detailed HTML report and update the accessibility summary.</t>
+  </si>
+  <si>
+    <t>The Employee List scan completes, detected issues are captured, and the scan results are available in the detailed report and summary.</t>
+  </si>
+  <si>
+    <t>TS12.1</t>
+  </si>
+  <si>
+    <t>Verify that the System Users page is scanned for accessibility violations.</t>
+  </si>
+  <si>
+    <t>Valid administrator credentials are available, and the administrator has access to User Management.</t>
+  </si>
+  <si>
+    <t>Administrator credentials; Admin → User Management/System Users page; configured axe-core accessibility rules.</t>
+  </si>
+  <si>
+    <t>1. Log in as Admin. 2. Navigate to Admin. 3. Open User Management and access the System Users page. 4. Verify that the target page is displayed. 5. Execute the axe-core accessibility scan. 6. Record violations, passes, and incomplete checks. 7. Generate the detailed HTML report and update the accessibility summary.</t>
+  </si>
+  <si>
+    <t>The System Users scan completes, detected issues are recorded, and the detailed report and summary are generated.</t>
+  </si>
+  <si>
+    <t>TS13.1</t>
+  </si>
+  <si>
+    <t>Verify that the Add User page is scanned for accessibility violations.</t>
+  </si>
+  <si>
+    <t>Valid administrator credentials are available, and the administrator can access the Add User form.</t>
+  </si>
+  <si>
+    <t>Administrator credentials; Admin → User Management → Add User page; configured axe-core accessibility rules.</t>
+  </si>
+  <si>
+    <t>1. Log in as Admin. 2. Navigate to Admin. 3. Open User Management. 4. Select Add User. 5. Verify that the Add User form is displayed. 6. Execute the axe-core accessibility scan. 7. Record violations, passes, and incomplete checks. 8. Generate the detailed HTML report and update the accessibility summary.</t>
+  </si>
+  <si>
+    <t>The Add User scan completes, detected issues are captured, and the detailed report and summary are generated.</t>
   </si>
 </sst>
 </file>
@@ -1508,7 +1679,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1531,11 +1702,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1583,9 +1765,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1595,13 +1774,25 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2057,35 +2248,75 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
+    <row r="10" spans="1:4" ht="28.8">
+      <c r="A10" s="10" t="s">
+        <v>403</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>413</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>404</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="28.8">
+      <c r="A11" s="10" t="s">
+        <v>405</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>414</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="28.8">
+      <c r="A12" s="10" t="s">
+        <v>407</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="28.8">
+      <c r="A13" s="10" t="s">
+        <v>409</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>416</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="28.8">
+      <c r="A14" s="10" t="s">
+        <v>411</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>417</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>412</v>
+      </c>
+      <c r="D14" s="11" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="1"/>
@@ -2184,13 +2415,14 @@
       <c r="D30" s="1"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA49C067-8F15-4F61-ABFB-E796688C4971}">
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="11.77734375" customWidth="1"/>
@@ -3418,94 +3650,94 @@
       </c>
     </row>
     <row r="47" spans="1:12" ht="43.2">
-      <c r="A47" s="18" t="s">
+      <c r="A47" s="17" t="s">
         <v>293</v>
       </c>
-      <c r="B47" s="19" t="s">
+      <c r="B47" s="18" t="s">
         <v>310</v>
       </c>
-      <c r="C47" s="20" t="s">
+      <c r="C47" s="19" t="s">
         <v>311</v>
       </c>
-      <c r="D47" s="21" t="s">
+      <c r="D47" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="E47" s="21" t="s">
+      <c r="E47" s="1" t="s">
         <v>313</v>
       </c>
-      <c r="F47" s="21" t="s">
+      <c r="F47" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="G47" s="21" t="s">
+      <c r="G47" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="H47" s="21" t="s">
+      <c r="H47" s="1" t="s">
         <v>316</v>
       </c>
     </row>
     <row r="48" spans="1:12" ht="43.2">
       <c r="A48" s="11"/>
-      <c r="B48" s="19" t="s">
+      <c r="B48" s="18" t="s">
         <v>331</v>
       </c>
       <c r="C48" s="11"/>
-      <c r="D48" s="17" t="s">
+      <c r="D48" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="E48" s="17" t="s">
+      <c r="E48" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="F48" s="17" t="s">
+      <c r="F48" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="G48" s="17" t="s">
+      <c r="G48" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="H48" s="17" t="s">
+      <c r="H48" s="1" t="s">
         <v>320</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="57.6">
       <c r="A49" s="11"/>
-      <c r="B49" s="19" t="s">
+      <c r="B49" s="18" t="s">
         <v>332</v>
       </c>
       <c r="C49" s="11"/>
-      <c r="D49" s="17" t="s">
+      <c r="D49" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="E49" s="17" t="s">
+      <c r="E49" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="F49" s="17" t="s">
+      <c r="F49" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="G49" s="17" t="s">
+      <c r="G49" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="H49" s="17" t="s">
+      <c r="H49" s="1" t="s">
         <v>325</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="43.2">
       <c r="A50" s="11"/>
-      <c r="B50" s="19" t="s">
+      <c r="B50" s="18" t="s">
         <v>333</v>
       </c>
       <c r="C50" s="11"/>
-      <c r="D50" s="17" t="s">
+      <c r="D50" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="E50" s="17" t="s">
+      <c r="E50" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="F50" s="17" t="s">
+      <c r="F50" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="G50" s="17" t="s">
+      <c r="G50" s="1" t="s">
         <v>329</v>
       </c>
-      <c r="H50" s="17" t="s">
+      <c r="H50" s="1" t="s">
         <v>330</v>
       </c>
     </row>
@@ -3513,201 +3745,201 @@
       <c r="A51" s="14" t="s">
         <v>296</v>
       </c>
-      <c r="B51" s="22" t="s">
+      <c r="B51" s="20" t="s">
         <v>376</v>
       </c>
       <c r="C51" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="D51" s="17" t="s">
+      <c r="D51" s="1" t="s">
         <v>334</v>
       </c>
-      <c r="E51" s="17" t="s">
+      <c r="E51" s="1" t="s">
         <v>335</v>
       </c>
-      <c r="F51" s="17" t="s">
+      <c r="F51" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="G51" s="17" t="s">
+      <c r="G51" s="1" t="s">
         <v>337</v>
       </c>
-      <c r="H51" s="17" t="s">
+      <c r="H51" s="1" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="43.2">
       <c r="A52" s="11"/>
-      <c r="B52" s="22" t="s">
+      <c r="B52" s="20" t="s">
         <v>377</v>
       </c>
       <c r="C52" s="11"/>
-      <c r="D52" s="17" t="s">
+      <c r="D52" s="1" t="s">
         <v>339</v>
       </c>
-      <c r="E52" s="17" t="s">
+      <c r="E52" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="F52" s="17" t="s">
+      <c r="F52" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="G52" s="17" t="s">
+      <c r="G52" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="H52" s="17" t="s">
+      <c r="H52" s="1" t="s">
         <v>343</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="43.2">
       <c r="A53" s="11"/>
-      <c r="B53" s="22" t="s">
+      <c r="B53" s="20" t="s">
         <v>378</v>
       </c>
       <c r="C53" s="11"/>
-      <c r="D53" s="17" t="s">
+      <c r="D53" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="E53" s="17" t="s">
+      <c r="E53" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="F53" s="17" t="s">
+      <c r="F53" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="G53" s="17" t="s">
+      <c r="G53" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="H53" s="17" t="s">
+      <c r="H53" s="1" t="s">
         <v>347</v>
       </c>
     </row>
     <row r="54" spans="1:8" ht="43.2">
       <c r="A54" s="11"/>
-      <c r="B54" s="22" t="s">
+      <c r="B54" s="20" t="s">
         <v>379</v>
       </c>
       <c r="C54" s="11"/>
-      <c r="D54" s="17" t="s">
+      <c r="D54" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="E54" s="17" t="s">
+      <c r="E54" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="F54" s="17" t="s">
+      <c r="F54" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="G54" s="17" t="s">
+      <c r="G54" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="H54" s="17" t="s">
+      <c r="H54" s="1" t="s">
         <v>352</v>
       </c>
     </row>
     <row r="55" spans="1:8" ht="43.2">
       <c r="A55" s="11"/>
-      <c r="B55" s="22" t="s">
+      <c r="B55" s="20" t="s">
         <v>380</v>
       </c>
       <c r="C55" s="11"/>
-      <c r="D55" s="17" t="s">
+      <c r="D55" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="E55" s="17" t="s">
+      <c r="E55" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="F55" s="17" t="s">
+      <c r="F55" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="G55" s="17" t="s">
+      <c r="G55" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="H55" s="17" t="s">
+      <c r="H55" s="1" t="s">
         <v>357</v>
       </c>
     </row>
     <row r="56" spans="1:8" ht="43.2">
       <c r="A56" s="11"/>
-      <c r="B56" s="22" t="s">
+      <c r="B56" s="20" t="s">
         <v>381</v>
       </c>
       <c r="C56" s="11"/>
-      <c r="D56" s="17" t="s">
+      <c r="D56" s="1" t="s">
         <v>358</v>
       </c>
-      <c r="E56" s="17" t="s">
+      <c r="E56" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="F56" s="17" t="s">
+      <c r="F56" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="G56" s="17" t="s">
+      <c r="G56" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="H56" s="17" t="s">
+      <c r="H56" s="1" t="s">
         <v>361</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="28.8">
       <c r="A57" s="11"/>
-      <c r="B57" s="22" t="s">
+      <c r="B57" s="20" t="s">
         <v>382</v>
       </c>
       <c r="C57" s="11"/>
-      <c r="D57" s="17" t="s">
+      <c r="D57" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="E57" s="17" t="s">
+      <c r="E57" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="F57" s="17" t="s">
+      <c r="F57" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="G57" s="17" t="s">
+      <c r="G57" s="1" t="s">
         <v>365</v>
       </c>
-      <c r="H57" s="17" t="s">
+      <c r="H57" s="1" t="s">
         <v>366</v>
       </c>
     </row>
     <row r="58" spans="1:8" ht="43.2">
       <c r="A58" s="11"/>
-      <c r="B58" s="22" t="s">
+      <c r="B58" s="20" t="s">
         <v>383</v>
       </c>
       <c r="C58" s="11"/>
-      <c r="D58" s="17" t="s">
+      <c r="D58" s="1" t="s">
         <v>367</v>
       </c>
-      <c r="E58" s="17" t="s">
+      <c r="E58" s="1" t="s">
         <v>368</v>
       </c>
-      <c r="F58" s="17" t="s">
+      <c r="F58" s="1" t="s">
         <v>369</v>
       </c>
-      <c r="G58" s="17" t="s">
+      <c r="G58" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="H58" s="17" t="s">
+      <c r="H58" s="1" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="59" spans="1:8" ht="28.8">
       <c r="A59" s="11"/>
-      <c r="B59" s="22" t="s">
+      <c r="B59" s="20" t="s">
         <v>384</v>
       </c>
       <c r="C59" s="11"/>
-      <c r="D59" s="17" t="s">
+      <c r="D59" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="E59" s="17" t="s">
+      <c r="E59" s="1" t="s">
         <v>373</v>
       </c>
-      <c r="F59" s="17" t="s">
+      <c r="F59" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="G59" s="17" t="s">
+      <c r="G59" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="H59" s="17" t="s">
+      <c r="H59" s="1" t="s">
         <v>375</v>
       </c>
     </row>
@@ -3715,70 +3947,200 @@
       <c r="A60" s="14" t="s">
         <v>299</v>
       </c>
-      <c r="B60" s="23" t="s">
+      <c r="B60" s="21" t="s">
         <v>400</v>
       </c>
       <c r="C60" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="D60" s="17" t="s">
+      <c r="D60" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="E60" s="17" t="s">
+      <c r="E60" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="F60" s="17" t="s">
+      <c r="F60" s="1" t="s">
         <v>387</v>
       </c>
-      <c r="G60" s="17" t="s">
+      <c r="G60" s="1" t="s">
         <v>388</v>
       </c>
-      <c r="H60" s="17" t="s">
+      <c r="H60" s="1" t="s">
         <v>389</v>
       </c>
     </row>
     <row r="61" spans="1:8" ht="43.2">
       <c r="A61" s="11"/>
-      <c r="B61" s="23" t="s">
+      <c r="B61" s="21" t="s">
         <v>401</v>
       </c>
       <c r="C61" s="11"/>
-      <c r="D61" s="17" t="s">
+      <c r="D61" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="E61" s="17" t="s">
+      <c r="E61" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="F61" s="17" t="s">
+      <c r="F61" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="G61" s="17" t="s">
+      <c r="G61" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="H61" s="17" t="s">
+      <c r="H61" s="1" t="s">
         <v>394</v>
       </c>
     </row>
     <row r="62" spans="1:8" ht="43.2">
       <c r="A62" s="11"/>
-      <c r="B62" s="23" t="s">
+      <c r="B62" s="21" t="s">
         <v>402</v>
       </c>
       <c r="C62" s="11"/>
-      <c r="D62" s="17" t="s">
+      <c r="D62" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="E62" s="17" t="s">
+      <c r="E62" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="F62" s="17" t="s">
+      <c r="F62" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="G62" s="17" t="s">
+      <c r="G62" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="H62" s="17" t="s">
+      <c r="H62" s="1" t="s">
         <v>399</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" ht="86.4">
+      <c r="A63" s="17" t="s">
+        <v>403</v>
+      </c>
+      <c r="B63" s="25" t="s">
+        <v>431</v>
+      </c>
+      <c r="C63" s="16" t="s">
+        <v>413</v>
+      </c>
+      <c r="D63" s="26" t="s">
+        <v>430</v>
+      </c>
+      <c r="E63" s="26" t="s">
+        <v>432</v>
+      </c>
+      <c r="F63" s="26" t="s">
+        <v>433</v>
+      </c>
+      <c r="G63" s="26" t="s">
+        <v>434</v>
+      </c>
+      <c r="H63" s="26" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" ht="86.4">
+      <c r="A64" s="17" t="s">
+        <v>405</v>
+      </c>
+      <c r="B64" s="25" t="s">
+        <v>437</v>
+      </c>
+      <c r="C64" s="16" t="s">
+        <v>414</v>
+      </c>
+      <c r="D64" s="26" t="s">
+        <v>436</v>
+      </c>
+      <c r="E64" s="26" t="s">
+        <v>438</v>
+      </c>
+      <c r="F64" s="26" t="s">
+        <v>439</v>
+      </c>
+      <c r="G64" s="26" t="s">
+        <v>440</v>
+      </c>
+      <c r="H64" s="26" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" ht="100.8">
+      <c r="A65" s="17" t="s">
+        <v>407</v>
+      </c>
+      <c r="B65" s="25" t="s">
+        <v>442</v>
+      </c>
+      <c r="C65" s="16" t="s">
+        <v>415</v>
+      </c>
+      <c r="D65" s="26" t="s">
+        <v>443</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="F65" s="26" t="s">
+        <v>445</v>
+      </c>
+      <c r="G65" s="26" t="s">
+        <v>446</v>
+      </c>
+      <c r="H65" s="26" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" ht="115.2">
+      <c r="A66" s="17" t="s">
+        <v>409</v>
+      </c>
+      <c r="B66" s="25" t="s">
+        <v>448</v>
+      </c>
+      <c r="C66" s="16" t="s">
+        <v>416</v>
+      </c>
+      <c r="D66" s="26" t="s">
+        <v>449</v>
+      </c>
+      <c r="E66" s="26" t="s">
+        <v>450</v>
+      </c>
+      <c r="F66" s="26" t="s">
+        <v>451</v>
+      </c>
+      <c r="G66" s="26" t="s">
+        <v>452</v>
+      </c>
+      <c r="H66" s="26" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" ht="100.8">
+      <c r="A67" s="17" t="s">
+        <v>411</v>
+      </c>
+      <c r="B67" s="25" t="s">
+        <v>454</v>
+      </c>
+      <c r="C67" s="16" t="s">
+        <v>417</v>
+      </c>
+      <c r="D67" s="26" t="s">
+        <v>455</v>
+      </c>
+      <c r="E67" s="26" t="s">
+        <v>456</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="G67" s="26" t="s">
+        <v>458</v>
+      </c>
+      <c r="H67" s="26" t="s">
+        <v>459</v>
       </c>
     </row>
   </sheetData>
@@ -3952,40 +4314,90 @@
         <v>307</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
+    <row r="10" spans="1:5" ht="57.6">
+      <c r="A10" s="10" t="s">
+        <v>403</v>
+      </c>
+      <c r="B10" s="24" t="s">
+        <v>413</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="57.6">
+      <c r="A11" s="10" t="s">
+        <v>405</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>421</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>422</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="57.6">
+      <c r="A12" s="10" t="s">
+        <v>407</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>415</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="72">
+      <c r="A13" s="10" t="s">
+        <v>409</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>416</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="72">
+      <c r="A14" s="10" t="s">
+        <v>411</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>417</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>429</v>
+      </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="7"/>

</xml_diff>